<commit_message>
finishing organizing constituent data
</commit_message>
<xml_diff>
--- a/data/raw_lab_data/GGRL_Valles_Caldera BER_NH.xlsx
+++ b/data/raw_lab_data/GGRL_Valles_Caldera BER_NH.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\hysteresis\data\raw_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\hysteresis\data\raw_lab_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{928C616A-5063-460F-B4FA-80246E8E70AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AA3E745-EE50-4601-9A97-6C3070074F3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="599" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="27036" yWindow="2112" windowWidth="17280" windowHeight="8880" tabRatio="599" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26493,7 +26493,7 @@
       <c r="N442" s="25"/>
       <c r="O442" s="25"/>
       <c r="P442" s="61">
-        <v>22.763000000000002</v>
+        <v>2.7629999999999999</v>
       </c>
       <c r="Q442" s="28">
         <v>0.2</v>

</xml_diff>